<commit_message>
Update notes w/ PEC info
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
+++ b/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/13_sctype_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84F1394B-A760-0941-B51F-B32ABB8F7E28}"/>
   <bookViews>
     <workbookView xWindow="37820" yWindow="1220" windowWidth="28040" windowHeight="17440" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="sctype_final-NOTES" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sctype_final-NOTES'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'sctype_final-NOTES'!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="123">
   <si>
     <t>cluster</t>
   </si>
@@ -339,13 +339,79 @@
   </si>
   <si>
     <t>NOTE</t>
+  </si>
+  <si>
+    <t>snDLPFC_PEC</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>L2.3.IT</t>
+  </si>
+  <si>
+    <t>L5.IT</t>
+  </si>
+  <si>
+    <t>L6b</t>
+  </si>
+  <si>
+    <t>L6.CT</t>
+  </si>
+  <si>
+    <t>L2.3.IT*</t>
+  </si>
+  <si>
+    <t>L5.IT/L2.3.IT/L5.6.NP*</t>
+  </si>
+  <si>
+    <t>L5.6.NP</t>
+  </si>
+  <si>
+    <t>Pax6</t>
+  </si>
+  <si>
+    <t>Vip</t>
+  </si>
+  <si>
+    <t>Pvalb</t>
+  </si>
+  <si>
+    <t>Lamp5.Lhx6/Lamp5</t>
+  </si>
+  <si>
+    <t>Sst</t>
+  </si>
+  <si>
+    <t>Chandelier</t>
+  </si>
+  <si>
+    <t>L2/3 * not the best Excit expression</t>
+  </si>
+  <si>
+    <t>Excit.L5</t>
+  </si>
+  <si>
+    <t>Inhib.Vip</t>
+  </si>
+  <si>
+    <t>Excit.L2_3.1</t>
+  </si>
+  <si>
+    <t>Excit.L2_3.2</t>
+  </si>
+  <si>
+    <t>Excit.L2_3.3</t>
+  </si>
+  <si>
+    <t>Excit.L4_5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -476,6 +542,12 @@
     <font>
       <sz val="12"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -869,7 +941,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -877,16 +949,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1220,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEA37F64-DEE8-C84A-AF9C-A45F7C1C524C}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
@@ -1234,10 +1296,10 @@
     <col min="9" max="9" width="15.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="15.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1272,21 +1334,24 @@
         <v>85</v>
       </c>
       <c r="L1" t="s">
+        <v>101</v>
+      </c>
+      <c r="M1" t="s">
         <v>99</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
       <c r="C2">
-        <v>46561.506809999999</v>
+        <v>94498.527289999998</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -1295,16 +1360,16 @@
         <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
         <v>8</v>
       </c>
       <c r="H2">
-        <v>253943.78350913001</v>
+        <v>516411.97841181501</v>
       </c>
       <c r="I2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J2" t="s">
         <v>8</v>
@@ -1314,18 +1379,21 @@
         <v>1</v>
       </c>
       <c r="L2" t="s">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="M2" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3">
-        <v>94498.527289999998</v>
+        <v>46561.506809999999</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -1334,16 +1402,16 @@
         <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
       </c>
       <c r="H3">
-        <v>516411.97841181501</v>
+        <v>253943.78350913001</v>
       </c>
       <c r="I3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J3" t="s">
         <v>8</v>
@@ -1353,10 +1421,13 @@
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="M3" t="s">
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>13</v>
       </c>
@@ -1391,18 +1462,21 @@
         <v>86</v>
       </c>
       <c r="L4" t="s">
+        <v>102</v>
+      </c>
+      <c r="M4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
         <v>38</v>
       </c>
       <c r="C5">
-        <v>11952.394829999999</v>
+        <v>46928.582920000001</v>
       </c>
       <c r="D5" t="s">
         <v>39</v>
@@ -1411,37 +1485,42 @@
         <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="H5">
-        <v>28117.8497458108</v>
+        <v>100317.098382357</v>
       </c>
       <c r="I5" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="J5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K5" t="b">
-        <f>D5=J5</f>
-        <v>1</v>
+        <v>23</v>
+      </c>
+      <c r="K5" t="s">
+        <v>89</v>
+      </c>
+      <c r="L5" t="s">
+        <v>103</v>
       </c>
       <c r="M5" t="s">
-        <v>87</v>
+        <v>119</v>
+      </c>
+      <c r="N5" t="s">
+        <v>116</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
         <v>38</v>
       </c>
       <c r="C6">
-        <v>4623.0345580000003</v>
+        <v>11952.394829999999</v>
       </c>
       <c r="D6" t="s">
         <v>39</v>
@@ -1450,16 +1529,16 @@
         <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="H6">
-        <v>16068.214590309901</v>
+        <v>28117.8497458108</v>
       </c>
       <c r="I6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J6" t="s">
         <v>39</v>
@@ -1469,13 +1548,16 @@
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>59</v>
+        <v>104</v>
       </c>
       <c r="M6" t="s">
-        <v>88</v>
+        <v>117</v>
+      </c>
+      <c r="N6" t="s">
+        <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -1509,19 +1591,25 @@
       <c r="K7" t="s">
         <v>89</v>
       </c>
+      <c r="L7" t="s">
+        <v>103</v>
+      </c>
       <c r="M7" t="s">
+        <v>120</v>
+      </c>
+      <c r="N7" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
         <v>38</v>
       </c>
       <c r="C8">
-        <v>761.70686350000005</v>
+        <v>4623.0345580000003</v>
       </c>
       <c r="D8" t="s">
         <v>39</v>
@@ -1530,16 +1618,16 @@
         <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="H8">
-        <v>2572.62219382998</v>
+        <v>16068.214590309901</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="J8" t="s">
         <v>39</v>
@@ -1549,21 +1637,24 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>65</v>
+        <v>105</v>
       </c>
       <c r="M8" t="s">
-        <v>95</v>
+        <v>59</v>
+      </c>
+      <c r="N8" t="s">
+        <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>38</v>
       </c>
       <c r="C9">
-        <v>46928.582920000001</v>
+        <v>3248.993226</v>
       </c>
       <c r="D9" t="s">
         <v>39</v>
@@ -1572,33 +1663,43 @@
         <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="G9" t="s">
-        <v>23</v>
+        <v>62</v>
       </c>
       <c r="H9">
-        <v>100317.098382357</v>
+        <v>9707.6033777966004</v>
       </c>
       <c r="I9" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="J9" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" t="s">
-        <v>89</v>
+        <v>39</v>
+      </c>
+      <c r="K9" t="b">
+        <f>D9=J9</f>
+        <v>1</v>
+      </c>
+      <c r="L9" t="s">
+        <v>106</v>
+      </c>
+      <c r="M9" t="s">
+        <v>62</v>
+      </c>
+      <c r="N9" t="s">
+        <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
         <v>38</v>
       </c>
       <c r="C10">
-        <v>549.06715540000005</v>
+        <v>3332.042692</v>
       </c>
       <c r="D10" t="s">
         <v>39</v>
@@ -1607,36 +1708,39 @@
         <v>40</v>
       </c>
       <c r="F10" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="G10" t="s">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="H10">
-        <v>1718.38000592344</v>
+        <v>7447.9189106358099</v>
       </c>
       <c r="I10" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
       <c r="J10" t="s">
-        <v>68</v>
+        <v>23</v>
       </c>
       <c r="K10" t="s">
-        <v>96</v>
+        <v>89</v>
+      </c>
+      <c r="L10" t="s">
+        <v>107</v>
       </c>
       <c r="M10" t="s">
-        <v>97</v>
+        <v>121</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>38</v>
       </c>
       <c r="C11">
-        <v>3332.042692</v>
+        <v>1329.846665</v>
       </c>
       <c r="D11" t="s">
         <v>39</v>
@@ -1645,16 +1749,16 @@
         <v>40</v>
       </c>
       <c r="F11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G11" t="s">
         <v>23</v>
       </c>
       <c r="H11">
-        <v>7447.9189106358099</v>
+        <v>2998.1614067282499</v>
       </c>
       <c r="I11" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J11" t="s">
         <v>23</v>
@@ -1662,16 +1766,25 @@
       <c r="K11" t="s">
         <v>89</v>
       </c>
+      <c r="L11" t="s">
+        <v>108</v>
+      </c>
+      <c r="M11" t="s">
+        <v>122</v>
+      </c>
+      <c r="N11" t="s">
+        <v>87</v>
+      </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
         <v>38</v>
       </c>
       <c r="C12">
-        <v>3248.993226</v>
+        <v>761.70686350000005</v>
       </c>
       <c r="D12" t="s">
         <v>39</v>
@@ -1680,16 +1793,16 @@
         <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="G12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H12">
-        <v>9707.6033777966004</v>
+        <v>2572.62219382998</v>
       </c>
       <c r="I12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="J12" t="s">
         <v>39</v>
@@ -1699,21 +1812,24 @@
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>62</v>
+        <v>109</v>
       </c>
       <c r="M12" t="s">
-        <v>88</v>
+        <v>65</v>
+      </c>
+      <c r="N12" t="s">
+        <v>95</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
         <v>38</v>
       </c>
       <c r="C13">
-        <v>1329.846665</v>
+        <v>549.06715540000005</v>
       </c>
       <c r="D13" t="s">
         <v>39</v>
@@ -1722,36 +1838,42 @@
         <v>40</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="G13" t="s">
-        <v>23</v>
+        <v>84</v>
       </c>
       <c r="H13">
-        <v>2998.1614067282499</v>
+        <v>1718.38000592344</v>
       </c>
       <c r="I13" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="J13" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="K13" t="s">
-        <v>89</v>
+        <v>96</v>
+      </c>
+      <c r="L13" t="s">
+        <v>110</v>
       </c>
       <c r="M13" t="s">
-        <v>87</v>
+        <v>84</v>
+      </c>
+      <c r="N13" t="s">
+        <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
         <v>67</v>
       </c>
       <c r="C14">
-        <v>6631.9579649999996</v>
+        <v>32834.18262</v>
       </c>
       <c r="D14" t="s">
         <v>68</v>
@@ -1760,37 +1882,39 @@
         <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="G14" t="s">
-        <v>70</v>
+        <v>23</v>
       </c>
       <c r="H14">
-        <v>17302.614439252699</v>
+        <v>80989.211091594305</v>
       </c>
       <c r="I14" t="s">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="J14" t="s">
-        <v>68</v>
-      </c>
-      <c r="K14" t="b">
-        <f>D14=J14</f>
-        <v>1</v>
+        <v>23</v>
+      </c>
+      <c r="K14" t="s">
+        <v>98</v>
       </c>
       <c r="L14" t="s">
-        <v>70</v>
+        <v>111</v>
+      </c>
+      <c r="M14" t="s">
+        <v>118</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B15" t="s">
         <v>67</v>
       </c>
       <c r="C15">
-        <v>32834.18262</v>
+        <v>6631.9579649999996</v>
       </c>
       <c r="D15" t="s">
         <v>68</v>
@@ -1799,25 +1923,32 @@
         <v>40</v>
       </c>
       <c r="F15" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G15" t="s">
-        <v>23</v>
+        <v>70</v>
       </c>
       <c r="H15">
-        <v>80989.211091594305</v>
+        <v>17302.614439252699</v>
       </c>
       <c r="I15" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="J15" t="s">
-        <v>23</v>
-      </c>
-      <c r="K15" t="s">
-        <v>98</v>
+        <v>68</v>
+      </c>
+      <c r="K15" t="b">
+        <f>D15=J15</f>
+        <v>1</v>
+      </c>
+      <c r="L15" t="s">
+        <v>112</v>
+      </c>
+      <c r="M15" t="s">
+        <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>74</v>
       </c>
@@ -1853,10 +1984,13 @@
         <v>1</v>
       </c>
       <c r="L16" t="s">
+        <v>113</v>
+      </c>
+      <c r="M16" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>19</v>
       </c>
@@ -1894,8 +2028,11 @@
       <c r="L17" t="s">
         <v>17</v>
       </c>
+      <c r="M17" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>22</v>
       </c>
@@ -1933,8 +2070,11 @@
       <c r="L18" t="s">
         <v>17</v>
       </c>
+      <c r="M18" t="s">
+        <v>21</v>
+      </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>77</v>
       </c>
@@ -1970,10 +2110,13 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
+        <v>114</v>
+      </c>
+      <c r="M19" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>82</v>
       </c>
@@ -2009,18 +2152,21 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
+        <v>115</v>
+      </c>
+      <c r="M20" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
         <v>26</v>
       </c>
       <c r="C21">
-        <v>114958.5073</v>
+        <v>159677.883</v>
       </c>
       <c r="D21" t="s">
         <v>23</v>
@@ -2029,16 +2175,16 @@
         <v>9</v>
       </c>
       <c r="F21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G21" t="s">
         <v>23</v>
       </c>
       <c r="H21">
-        <v>747160.65919662802</v>
+        <v>1089890.18814854</v>
       </c>
       <c r="I21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J21" t="s">
         <v>23</v>
@@ -2050,16 +2196,19 @@
       <c r="L21" t="s">
         <v>23</v>
       </c>
+      <c r="M21" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
       </c>
       <c r="C22">
-        <v>159677.883</v>
+        <v>114958.5073</v>
       </c>
       <c r="D22" t="s">
         <v>23</v>
@@ -2068,16 +2217,16 @@
         <v>9</v>
       </c>
       <c r="F22" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G22" t="s">
         <v>23</v>
       </c>
       <c r="H22">
-        <v>1089890.18814854</v>
+        <v>747160.65919662802</v>
       </c>
       <c r="I22" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="J22" t="s">
         <v>23</v>
@@ -2089,8 +2238,11 @@
       <c r="L22" t="s">
         <v>23</v>
       </c>
+      <c r="M22" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -2125,11 +2277,11 @@
         <f>D23=J23</f>
         <v>1</v>
       </c>
-      <c r="L23" t="s">
-        <v>23</v>
+      <c r="M23" t="s">
+        <v>29</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>32</v>
       </c>
@@ -2167,10 +2319,18 @@
       <c r="L24" t="s">
         <v>34</v>
       </c>
+      <c r="M24" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M1" xr:uid="{FEA37F64-DEE8-C84A-AF9C-A45F7C1C524C}"/>
-  <conditionalFormatting sqref="K2:L24 M5:M8 M10 M12:M13">
+  <autoFilter ref="A1:N1" xr:uid="{FEA37F64-DEE8-C84A-AF9C-A45F7C1C524C}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N24">
+      <sortCondition ref="F1:F24"/>
+    </sortState>
+  </autoFilter>
+  <phoneticPr fontId="18" type="noConversion"/>
+  <conditionalFormatting sqref="N10 N12:N13 K23 K24:M24 K2:M21 N5:N8 K22:L22 M22:M23">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>

</xml_diff>

<commit_message>
Label Oligo.3 as choird plexis
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
+++ b/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/13_sctype_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84F1394B-A760-0941-B51F-B32ABB8F7E28}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E074096-B23B-814D-AC67-5684A2F22D9E}"/>
   <bookViews>
-    <workbookView xWindow="37820" yWindow="1220" windowWidth="28040" windowHeight="17440" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
   </bookViews>
   <sheets>
     <sheet name="sctype_final-NOTES" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="124">
   <si>
     <t>cluster</t>
   </si>
@@ -405,6 +405,9 @@
   </si>
   <si>
     <t>Excit.L4_5</t>
+  </si>
+  <si>
+    <t>choird_plexis</t>
   </si>
 </sst>
 </file>
@@ -1938,7 +1941,7 @@
         <v>68</v>
       </c>
       <c r="K15" t="b">
-        <f>D15=J15</f>
+        <f t="shared" ref="K15:K24" si="0">D15=J15</f>
         <v>1</v>
       </c>
       <c r="L15" t="s">
@@ -1980,7 +1983,7 @@
         <v>68</v>
       </c>
       <c r="K16" t="b">
-        <f>D16=J16</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L16" t="s">
@@ -2022,7 +2025,7 @@
         <v>17</v>
       </c>
       <c r="K17" t="b">
-        <f>D17=J17</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L17" t="s">
@@ -2064,7 +2067,7 @@
         <v>17</v>
       </c>
       <c r="K18" t="b">
-        <f>D18=J18</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L18" t="s">
@@ -2106,7 +2109,7 @@
         <v>68</v>
       </c>
       <c r="K19" t="b">
-        <f>D19=J19</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L19" t="s">
@@ -2148,7 +2151,7 @@
         <v>68</v>
       </c>
       <c r="K20" t="b">
-        <f>D20=J20</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L20" t="s">
@@ -2190,7 +2193,7 @@
         <v>23</v>
       </c>
       <c r="K21" t="b">
-        <f>D21=J21</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L21" t="s">
@@ -2232,7 +2235,7 @@
         <v>23</v>
       </c>
       <c r="K22" t="b">
-        <f>D22=J22</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L22" t="s">
@@ -2274,11 +2277,11 @@
         <v>23</v>
       </c>
       <c r="K23" t="b">
-        <f>D23=J23</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>29</v>
+        <v>123</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">
@@ -2313,7 +2316,7 @@
         <v>34</v>
       </c>
       <c r="K24" t="b">
-        <f>D24=J24</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="L24" t="s">
@@ -2330,7 +2333,7 @@
     </sortState>
   </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>
-  <conditionalFormatting sqref="N10 N12:N13 K23 K24:M24 K2:M21 N5:N8 K22:L22 M22:M23">
+  <conditionalFormatting sqref="K2:M21 N5:N8 N10 N12:N13 K22:L22 M22:M23 K23 K24:M24">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>TRUE</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update L4 to LD for "lamina dissecans"
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
+++ b/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/13_sctype_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E074096-B23B-814D-AC67-5684A2F22D9E}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{770F0E78-C919-F74C-A308-764ABD21CF11}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
+    <workbookView xWindow="480" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
   </bookViews>
   <sheets>
     <sheet name="sctype_final-NOTES" sheetId="1" r:id="rId1"/>
@@ -323,9 +323,6 @@
     <t>L2/3</t>
   </si>
   <si>
-    <t>L4/5/6</t>
-  </si>
-  <si>
     <t>Excit/Inhib</t>
   </si>
   <si>
@@ -395,19 +392,22 @@
     <t>Inhib.Vip</t>
   </si>
   <si>
-    <t>Excit.L2_3.1</t>
-  </si>
-  <si>
-    <t>Excit.L2_3.2</t>
-  </si>
-  <si>
-    <t>Excit.L2_3.3</t>
-  </si>
-  <si>
     <t>Excit.L4_5</t>
   </si>
   <si>
     <t>choird_plexis</t>
+  </si>
+  <si>
+    <t>Excit.L2_5.1</t>
+  </si>
+  <si>
+    <t>Excit.L2</t>
+  </si>
+  <si>
+    <t>Excit.L2_5.2</t>
+  </si>
+  <si>
+    <t>L4/5/6, ETV1 ~ L5a</t>
   </si>
 </sst>
 </file>
@@ -1337,13 +1337,13 @@
         <v>85</v>
       </c>
       <c r="L1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N1" t="s">
         <v>99</v>
-      </c>
-      <c r="N1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -1465,7 +1465,7 @@
         <v>86</v>
       </c>
       <c r="L4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M4" t="s">
         <v>15</v>
@@ -1506,13 +1506,13 @@
         <v>89</v>
       </c>
       <c r="L5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="N5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -1551,10 +1551,10 @@
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="N6" t="s">
         <v>87</v>
@@ -1595,10 +1595,10 @@
         <v>89</v>
       </c>
       <c r="L7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N7" t="s">
         <v>94</v>
@@ -1640,7 +1640,7 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M8" t="s">
         <v>59</v>
@@ -1685,7 +1685,7 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M9" t="s">
         <v>62</v>
@@ -1729,10 +1729,10 @@
         <v>89</v>
       </c>
       <c r="L10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -1770,10 +1770,10 @@
         <v>89</v>
       </c>
       <c r="L11" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M11" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="N11" t="s">
         <v>87</v>
@@ -1815,13 +1815,13 @@
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="M12" t="s">
         <v>65</v>
       </c>
       <c r="N12" t="s">
-        <v>95</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1856,16 +1856,16 @@
         <v>68</v>
       </c>
       <c r="K13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M13" t="s">
         <v>84</v>
       </c>
       <c r="N13" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
@@ -1900,13 +1900,13 @@
         <v>23</v>
       </c>
       <c r="K14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -1945,7 +1945,7 @@
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M15" t="s">
         <v>70</v>
@@ -1987,7 +1987,7 @@
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M16" t="s">
         <v>73</v>
@@ -2113,7 +2113,7 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M19" t="s">
         <v>76</v>
@@ -2155,7 +2155,7 @@
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M20" t="s">
         <v>81</v>
@@ -2281,7 +2281,7 @@
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Update Excit_L4_5 annotation, update colors too
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
+++ b/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/13_sctype_final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/louise.huuki/Library/CloudStorage/OneDrive-LieberInstituteforBrainDevelopment/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/13_sctype_final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{6C2E3B46-881E-104E-9C6F-4068EED76B5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{770F0E78-C919-F74C-A308-764ABD21CF11}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BC3396-DDB2-804D-A920-2199FB97D7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17420" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
   </bookViews>
   <sheets>
     <sheet name="sctype_final-NOTES" sheetId="1" r:id="rId1"/>
@@ -386,15 +386,9 @@
     <t>L2/3 * not the best Excit expression</t>
   </si>
   <si>
-    <t>Excit.L5</t>
-  </si>
-  <si>
     <t>Inhib.Vip</t>
   </si>
   <si>
-    <t>Excit.L4_5</t>
-  </si>
-  <si>
     <t>choird_plexis</t>
   </si>
   <si>
@@ -408,6 +402,12 @@
   </si>
   <si>
     <t>L4/5/6, ETV1 ~ L5a</t>
+  </si>
+  <si>
+    <t>Excit.L5.1</t>
+  </si>
+  <si>
+    <t>Excit.L5.2</t>
   </si>
 </sst>
 </file>
@@ -1509,7 +1509,7 @@
         <v>102</v>
       </c>
       <c r="M5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="N5" t="s">
         <v>115</v>
@@ -1554,7 +1554,7 @@
         <v>103</v>
       </c>
       <c r="M6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="N6" t="s">
         <v>87</v>
@@ -1598,7 +1598,7 @@
         <v>102</v>
       </c>
       <c r="M7" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N7" t="s">
         <v>94</v>
@@ -1732,7 +1732,7 @@
         <v>106</v>
       </c>
       <c r="M10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -1773,7 +1773,7 @@
         <v>107</v>
       </c>
       <c r="M11" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="N11" t="s">
         <v>87</v>
@@ -1821,7 +1821,7 @@
         <v>65</v>
       </c>
       <c r="N12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1906,7 +1906,7 @@
         <v>110</v>
       </c>
       <c r="M14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -2281,7 +2281,7 @@
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Change Neun broad cell types to Inhib
</commit_message>
<xml_diff>
--- a/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
+++ b/processed-data/04_snRNA-seq/13_sctype_final/sctype_final-NOTES.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/louise.huuki/Library/CloudStorage/OneDrive-LieberInstituteforBrainDevelopment/LIBD_code/LFF_spatial_ERC/processed-data/04_snRNA-seq/13_sctype_final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/0n/5c96lsrn29jggjs673wwfmr00000gn/T/ch.sudo.cyberduck/editor-d6d7eaa6-642d-4271-ba48-6f9f0a048187/2cf5724336fb92b56101bb96f8833a44/1303047750/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BC3396-DDB2-804D-A920-2199FB97D7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37492B2-9728-434E-B48F-7056E14E14FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17420" xr2:uid="{29A9A955-D5B8-1042-8754-9C10FC181668}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="123">
   <si>
     <t>cluster</t>
   </si>
@@ -273,9 +273,6 @@
   </si>
   <si>
     <t>Mature neurons</t>
-  </si>
-  <si>
-    <t>Neu</t>
   </si>
   <si>
     <t>Neu.1</t>
@@ -1322,28 +1319,28 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H1" t="s">
         <v>90</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>91</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>92</v>
       </c>
-      <c r="J1" t="s">
-        <v>93</v>
-      </c>
       <c r="K1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M1" t="s">
+        <v>97</v>
+      </c>
+      <c r="N1" t="s">
         <v>98</v>
-      </c>
-      <c r="N1" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -1462,10 +1459,10 @@
         <v>53</v>
       </c>
       <c r="K4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M4" t="s">
         <v>15</v>
@@ -1503,16 +1500,16 @@
         <v>23</v>
       </c>
       <c r="K5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="N5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -1551,13 +1548,13 @@
         <v>1</v>
       </c>
       <c r="L6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="M6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="N6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -1592,16 +1589,16 @@
         <v>23</v>
       </c>
       <c r="K7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -1640,13 +1637,13 @@
         <v>1</v>
       </c>
       <c r="L8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M8" t="s">
         <v>59</v>
       </c>
       <c r="N8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -1685,13 +1682,13 @@
         <v>1</v>
       </c>
       <c r="L9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M9" t="s">
         <v>62</v>
       </c>
       <c r="N9" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -1726,13 +1723,13 @@
         <v>23</v>
       </c>
       <c r="K10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -1767,16 +1764,16 @@
         <v>23</v>
       </c>
       <c r="K11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="M11" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -1815,13 +1812,13 @@
         <v>1</v>
       </c>
       <c r="L12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="M12" t="s">
         <v>65</v>
       </c>
       <c r="N12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -1844,28 +1841,28 @@
         <v>64</v>
       </c>
       <c r="G13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H13">
         <v>1718.38000592344</v>
       </c>
       <c r="I13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J13" t="s">
         <v>68</v>
       </c>
       <c r="K13" t="s">
+        <v>94</v>
+      </c>
+      <c r="L13" t="s">
+        <v>108</v>
+      </c>
+      <c r="M13" t="s">
+        <v>83</v>
+      </c>
+      <c r="N13" t="s">
         <v>95</v>
-      </c>
-      <c r="L13" t="s">
-        <v>109</v>
-      </c>
-      <c r="M13" t="s">
-        <v>84</v>
-      </c>
-      <c r="N13" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
@@ -1900,13 +1897,13 @@
         <v>23</v>
       </c>
       <c r="K14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L14" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -1945,7 +1942,7 @@
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M15" t="s">
         <v>70</v>
@@ -1987,7 +1984,7 @@
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="M16" t="s">
         <v>73</v>
@@ -2088,13 +2085,13 @@
         <v>3533.6350010000001</v>
       </c>
       <c r="D19" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E19" t="s">
         <v>40</v>
       </c>
       <c r="F19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G19" t="s">
         <v>76</v>
@@ -2110,10 +2107,10 @@
       </c>
       <c r="K19" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M19" t="s">
         <v>76</v>
@@ -2121,7 +2118,7 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
         <v>78</v>
@@ -2130,35 +2127,35 @@
         <v>1261.221855</v>
       </c>
       <c r="D20" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E20" t="s">
         <v>40</v>
       </c>
       <c r="F20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H20">
         <v>6318.0305069945398</v>
       </c>
       <c r="I20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J20" t="s">
         <v>68</v>
       </c>
       <c r="K20" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L20" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
@@ -2281,7 +2278,7 @@
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>